<commit_message>
Margin calculator: number from 268, real clickable source links, 950 exchange rate, exact original font/color/format
</commit_message>
<xml_diff>
--- a/data/마진계산기_템플릿.xlsx
+++ b/data/마진계산기_템플릿.xlsx
@@ -21,13 +21,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="78">
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <rFont val="Cambria"/>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="70">
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
@@ -35,7 +34,6 @@
     </r>
     <r>
       <rPr>
-        <b val="true"/>
         <sz val="11"/>
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
@@ -44,9 +42,8 @@
     </r>
     <r>
       <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <rFont val="Cambria"/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
@@ -63,8 +60,8 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
@@ -74,9 +71,9 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Cambria"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
@@ -85,8 +82,8 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
@@ -95,9 +92,9 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Cambria"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
@@ -137,8 +134,8 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
@@ -148,9 +145,9 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Cambria"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
@@ -159,8 +156,8 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
@@ -169,9 +166,9 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Cambria"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
@@ -185,8 +182,8 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
@@ -195,9 +192,9 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Cambria"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
@@ -208,8 +205,8 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
@@ -219,9 +216,9 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Cambria"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
@@ -231,8 +228,8 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
@@ -243,8 +240,8 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
@@ -254,9 +251,9 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Cambria"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
@@ -265,8 +262,8 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
@@ -275,9 +272,9 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Cambria"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
@@ -286,8 +283,8 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
@@ -296,9 +293,9 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Cambria"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
@@ -420,15 +417,9 @@
     <t xml:space="preserve">선크림・로션</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">공식판매처</t>
-    </r>
+    <t xml:space="preserve">바로가기</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -437,16 +428,33 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(jolse.com, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">원출처 </t>
+      <t xml:space="preserve">002. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그린토마토 딥포어 클린 엔자임 파우더워시</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">320001641</t>
+  </si>
+  <si>
+    <t xml:space="preserve">113035</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">グリーントマト ディープポア クリーン エンザイム パウダーウォッシュ </t>
     </r>
     <r>
       <rPr>
@@ -456,8 +464,23 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">celimax.co.kr)</t>
-    </r>
+      <t xml:space="preserve">50g / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">韓国化粧品</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Sung Boon Editor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">세안 파우더</t>
   </si>
   <si>
     <r>
@@ -468,33 +491,16 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">002. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">그린토마토 딥포어 클린 엔자임 파우더워시</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">320001641</t>
-  </si>
-  <si>
-    <t xml:space="preserve">113035</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">グリーントマト ディープポア クリーン エンザイム パウダーウォッシュ </t>
+      <t xml:space="preserve">003. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">데미지 테라피 노워시 트리트먼트 </t>
     </r>
     <r>
       <rPr>
@@ -504,33 +510,24 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">50g / </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">韓国化粧品</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Sung Boon Editor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">세안 파우더</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">공식몰</t>
+      <t xml:space="preserve">EX(Due Rose)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">320001781</t>
+  </si>
+  <si>
+    <t xml:space="preserve">109569</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">【オリヤン１位】ダメージセラピーノーウォッシュトリートメント</t>
     </r>
     <r>
       <rPr>
@@ -540,8 +537,23 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(sungboon.com)</t>
-    </r>
+      <t xml:space="preserve">EX 250ml 2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">種</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">GROWUS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">씻어내지 않는 트리트먼트</t>
   </si>
   <si>
     <r>
@@ -552,16 +564,16 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">003. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">데미지 테라피 노워시 트리트먼트 </t>
+      <t xml:space="preserve">004. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그린티 히알루론산 미스트 </t>
     </r>
     <r>
       <rPr>
@@ -571,24 +583,24 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">EX(Due Rose)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">320001781</t>
-  </si>
-  <si>
-    <t xml:space="preserve">109569</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">【オリヤン１位】ダメージセラピーノーウォッシュトリートメント</t>
+      <t xml:space="preserve">150mL</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">320001634</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20802</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">グリーンティー ヒアルロン酸 ミスト</t>
     </r>
     <r>
       <rPr>
@@ -598,34 +610,25 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">EX 250ml 2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">種</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">GROWUS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">씻어내지 않는 트리트먼트</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">공식몰</t>
-    </r>
+      <t xml:space="preserve">150ml1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">本</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">イニスフリー</t>
+  </si>
+  <si>
+    <t xml:space="preserve">보습 미스트</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -634,10 +637,17 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(growus.kr)</t>
-    </r>
-  </si>
-  <si>
+      <t xml:space="preserve">005. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">단백질 본드 모이스트 앰플 에센스 </t>
+    </r>
     <r>
       <rPr>
         <sz val="11"/>
@@ -646,16 +656,24 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">004. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">그린티 히알루론산 미스트 </t>
+      <t xml:space="preserve">145ml</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">320001778</t>
+  </si>
+  <si>
+    <t xml:space="preserve">58304</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">プロテインボンド アンプル ヘアエッセンス </t>
     </r>
     <r>
       <rPr>
@@ -665,25 +683,25 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">150mL</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">320001634</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20802</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">グリーンティー ヒアルロン酸 ミスト</t>
-    </r>
+      <t xml:space="preserve">145ml </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">洗い流さないトリートメント 韓国ヘアケア</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">ヘアプラス</t>
+  </si>
+  <si>
+    <t xml:space="preserve">헤어 오일</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -692,33 +710,16 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">150ml1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">本</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">イニスフリー</t>
-  </si>
-  <si>
-    <t xml:space="preserve">보습 미스트</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">공식몰</t>
+      <t xml:space="preserve">006. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">닥터 마스크 시카 </t>
     </r>
     <r>
       <rPr>
@@ -728,10 +729,34 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(innisfree.com)</t>
-    </r>
-  </si>
-  <si>
+      <t xml:space="preserve">5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">매입</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">320001628</t>
+  </si>
+  <si>
+    <t xml:space="preserve">66535</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ドクターマスク シカ </t>
+    </r>
     <r>
       <rPr>
         <sz val="11"/>
@@ -740,17 +765,25 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">005. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">단백질 본드 모이스트 앰플 에센스 </t>
-    </r>
+      <t xml:space="preserve">5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">枚</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">ロベクチン</t>
+  </si>
+  <si>
+    <t xml:space="preserve">마스크 팩</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -759,24 +792,16 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">145ml</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">320001778</t>
-  </si>
-  <si>
-    <t xml:space="preserve">58304</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">プロテインボンド アンプル ヘアエッセンス </t>
+      <t xml:space="preserve">007. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">가히 멀티밤 리필키트 </t>
     </r>
     <r>
       <rPr>
@@ -786,33 +811,33 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">145ml </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">洗い流さないトリートメント 韓国ヘアケア</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">ヘアプラス</t>
-  </si>
-  <si>
-    <t xml:space="preserve">헤어 오일</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">공식몰</t>
+      <t xml:space="preserve">(9g) 2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">320001625</t>
+  </si>
+  <si>
+    <t xml:space="preserve">103034</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">マルチバームおかわりキット </t>
     </r>
     <r>
       <rPr>
@@ -822,176 +847,6 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(hairplus.co.kr)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">006. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">닥터 마스크 시카 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">매입</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">320001628</t>
-  </si>
-  <si>
-    <t xml:space="preserve">66535</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">ドクターマスク シカ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">枚</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">ロベクチン</t>
-  </si>
-  <si>
-    <t xml:space="preserve">마스크 팩</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">공식몰</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(rovectin.co.kr)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">007. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">가히 멀티밤 리필키트 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(9g) 2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">개</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">320001625</t>
-  </si>
-  <si>
-    <t xml:space="preserve">103034</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">マルチバームおかわりキット </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
       <t xml:space="preserve">9g x 2</t>
     </r>
     <r>
@@ -1013,58 +868,28 @@
   <si>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">공식몰</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(kahi.shop)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">파란 글씨 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Cambria"/>
+        <b val="true"/>
+        <sz val="12"/>
+        <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">= </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">직접 입력 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Cambria"/>
+      <t xml:space="preserve">KSE </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">요율표</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
@@ -1072,18 +897,18 @@
     </r>
     <r>
       <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">무게・국내구매가・환율・수수료율・목표마진율 등 수정 가능</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Cambria"/>
+        <b val="true"/>
+        <sz val="12"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">해상</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
@@ -1093,168 +918,65 @@
   <si>
     <r>
       <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">검정 글씨 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Cambria"/>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">배송비</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">= </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">자동 계산 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Cambria"/>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">엔화</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">배송비</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">(</t>
     </r>
     <r>
       <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">수식</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Cambria"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <rFont val="Cambria"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">KSE </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">요율표</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <rFont val="Cambria"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">해상</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <rFont val="Cambria"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">배송비</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <rFont val="Cambria"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">엔화</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <rFont val="Cambria"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">배송비</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <rFont val="Cambria"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
         <b val="true"/>
         <sz val="11"/>
         <rFont val="Noto Sans CJK SC"/>
@@ -1266,7 +988,7 @@
       <rPr>
         <b val="true"/>
         <sz val="11"/>
-        <rFont val="Cambria"/>
+        <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
@@ -1278,14 +1000,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="\₩#,##0"/>
-    <numFmt numFmtId="166" formatCode="\¥#,##0"/>
-    <numFmt numFmtId="167" formatCode="0%"/>
-    <numFmt numFmtId="168" formatCode="0.00%"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* \-_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="\₩#,##0_);&quot;(₩&quot;#,##0\)"/>
+    <numFmt numFmtId="167" formatCode="[$¥-411]#,##0"/>
+    <numFmt numFmtId="168" formatCode="\¥#,##0"/>
+    <numFmt numFmtId="169" formatCode="_-* #,##0_-;\-* #,##0_-;_-* \-_-;_-@_-"/>
+    <numFmt numFmtId="170" formatCode="0%"/>
+    <numFmt numFmtId="171" formatCode="\₩#,##0"/>
+    <numFmt numFmtId="172" formatCode="0.00%"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1309,30 +1035,28 @@
       <family val="0"/>
     </font>
     <font>
+      <sz val="11"/>
+      <name val="맑은 고딕"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Noto Sans CJK SC"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="11"/>
-      <name val="Cambria"/>
+      <color rgb="FF000000"/>
+      <name val="맑은 고딕"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="11"/>
-      <name val="Noto Sans CJK SC"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Cambria"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF000000"/>
       <name val="Noto Sans CJK SC"/>
       <family val="2"/>
     </font>
@@ -1343,47 +1067,16 @@
       <family val="2"/>
     </font>
     <font>
+      <u val="single"/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Cambria"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Cambria"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FF0563C1"/>
       <name val="Noto Sans CJK SC"/>
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
-      <name val="Cambria"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Noto Sans CJK SC"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Cambria"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <b val="true"/>
       <sz val="12"/>
-      <name val="Cambria"/>
+      <name val="맑은 고딕"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -1392,6 +1085,19 @@
       <sz val="12"/>
       <name val="Noto Sans CJK SC"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <name val="Noto Sans CJK SC"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <name val="맑은 고딕"/>
+      <family val="0"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1403,8 +1109,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF4472C4"/>
-        <bgColor rgb="FF666699"/>
+        <fgColor rgb="FFDCEDD5"/>
+        <bgColor rgb="FFCCFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -1417,18 +1123,10 @@
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
-      <left style="thin">
-        <color rgb="FFB7B7B7"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB7B7B7"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB7B7B7"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB7B7B7"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -1494,43 +1192,43 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1559,7 +1257,7 @@
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFB7B7B7"/>
+      <rgbColor rgb="FFC0C0C0"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
@@ -1567,7 +1265,7 @@
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FF0563C1"/>
       <rgbColor rgb="FFCCCCFF"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
@@ -1579,13 +1277,13 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFDCEDD5"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF4472C4"/>
+      <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
@@ -1786,26 +1484,27 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:V13"/>
+  <dimension ref="A1:V9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="16" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="19" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="44.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="11.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="6.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="11.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="10.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="13.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="13.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="16.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="11.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="19" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="10.62"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1813,7 +1512,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1881,9 +1580,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="n">
-        <v>1</v>
+        <v>268</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>23</v>
@@ -1906,57 +1605,57 @@
       <c r="H3" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="J3" s="8" t="n">
+      <c r="J3" s="9" t="n">
         <v>0.75</v>
       </c>
-      <c r="K3" s="9" t="n">
+      <c r="K3" s="10" t="n">
         <v>17600</v>
       </c>
-      <c r="L3" s="10" t="n">
+      <c r="L3" s="11" t="n">
         <f aca="false">(K3+P3+Q3+R3-K3/11)/(1-V3-O3)/N3*100</f>
-        <v>3864.96913580247</v>
-      </c>
-      <c r="M3" s="11" t="n">
+        <v>3661.54970760234</v>
+      </c>
+      <c r="M3" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="N3" s="8" t="n">
-        <v>900</v>
-      </c>
-      <c r="O3" s="12" t="n">
+      <c r="N3" s="13" t="n">
+        <v>950</v>
+      </c>
+      <c r="O3" s="14" t="n">
         <v>0.16</v>
       </c>
-      <c r="P3" s="9" t="n">
+      <c r="P3" s="10" t="n">
         <v>2080</v>
       </c>
-      <c r="Q3" s="13" t="n">
+      <c r="Q3" s="15" t="n">
         <f aca="false">VLOOKUP(J3,kse요율!$A$4:$C$28,3,0)</f>
         <v>6800</v>
       </c>
-      <c r="R3" s="9" t="n">
+      <c r="R3" s="15" t="n">
         <v>165</v>
       </c>
-      <c r="S3" s="13" t="n">
+      <c r="S3" s="15" t="n">
         <f aca="false">(L3+M3)*N3/100*(1-O3)-K3-P3-Q3-R3</f>
         <v>2574.16666666667</v>
       </c>
-      <c r="T3" s="13" t="n">
+      <c r="T3" s="15" t="n">
         <f aca="false">ROUNDUP((K3+P3)*0.090909,0)</f>
         <v>1790</v>
       </c>
-      <c r="U3" s="13" t="n">
+      <c r="U3" s="15" t="n">
         <f aca="false">S3+T3</f>
         <v>4364.16666666667</v>
       </c>
-      <c r="V3" s="14" t="n">
+      <c r="V3" s="16" t="n">
         <v>0.12</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="n">
-        <v>2</v>
+        <v>269</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>23</v>
@@ -1979,430 +1678,429 @@
       <c r="H4" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="I4" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="J4" s="8" t="n">
+      <c r="I4" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="J4" s="9" t="n">
         <v>0.5</v>
       </c>
-      <c r="K4" s="9" t="n">
+      <c r="K4" s="10" t="n">
         <v>12900</v>
       </c>
-      <c r="L4" s="10" t="n">
+      <c r="L4" s="11" t="n">
         <f aca="false">(K4+P4+Q4+R4-K4/11)/(1-V4-O4)/N4*100</f>
-        <v>3066.70875420875</v>
-      </c>
-      <c r="M4" s="11" t="n">
+        <v>2905.30303030303</v>
+      </c>
+      <c r="M4" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="N4" s="8" t="n">
-        <v>900</v>
-      </c>
-      <c r="O4" s="12" t="n">
+      <c r="N4" s="13" t="n">
+        <v>950</v>
+      </c>
+      <c r="O4" s="14" t="n">
         <v>0.16</v>
       </c>
-      <c r="P4" s="9" t="n">
+      <c r="P4" s="10" t="n">
         <v>2080</v>
       </c>
-      <c r="Q4" s="13" t="n">
+      <c r="Q4" s="15" t="n">
         <f aca="false">VLOOKUP(J4,kse요율!$A$4:$C$28,3,0)</f>
         <v>5900</v>
       </c>
-      <c r="R4" s="9" t="n">
+      <c r="R4" s="15" t="n">
         <v>165</v>
       </c>
-      <c r="S4" s="13" t="n">
+      <c r="S4" s="15" t="n">
         <f aca="false">(L4+M4)*N4/100*(1-O4)-K4-P4-Q4-R4</f>
         <v>2139.31818181819</v>
       </c>
-      <c r="T4" s="13" t="n">
+      <c r="T4" s="15" t="n">
         <f aca="false">ROUNDUP((K4+P4)*0.090909,0)</f>
         <v>1362</v>
       </c>
-      <c r="U4" s="13" t="n">
+      <c r="U4" s="15" t="n">
         <f aca="false">S4+T4</f>
         <v>3501.31818181819</v>
       </c>
-      <c r="V4" s="14" t="n">
+      <c r="V4" s="16" t="n">
         <v>0.12</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="n">
-        <v>3</v>
+        <v>270</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>23</v>
       </c>
       <c r="C5" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="F5" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="G5" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="H5" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="H5" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="J5" s="8" t="n">
+      <c r="I5" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="J5" s="9" t="n">
         <v>0.75</v>
       </c>
-      <c r="K5" s="9" t="n">
+      <c r="K5" s="10" t="n">
         <v>20800</v>
       </c>
-      <c r="L5" s="10" t="n">
+      <c r="L5" s="11" t="n">
         <f aca="false">(K5+P5+Q5+R5-K5/11)/(1-V5-O5)/N5*100</f>
-        <v>4313.90291806958</v>
-      </c>
-      <c r="M5" s="11" t="n">
+        <v>4086.85539606592</v>
+      </c>
+      <c r="M5" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="N5" s="8" t="n">
-        <v>900</v>
-      </c>
-      <c r="O5" s="12" t="n">
+      <c r="N5" s="13" t="n">
+        <v>950</v>
+      </c>
+      <c r="O5" s="14" t="n">
         <v>0.16</v>
       </c>
-      <c r="P5" s="9" t="n">
+      <c r="P5" s="10" t="n">
         <v>2080</v>
       </c>
-      <c r="Q5" s="13" t="n">
+      <c r="Q5" s="15" t="n">
         <f aca="false">VLOOKUP(J5,kse요율!$A$4:$C$28,3,0)</f>
         <v>6800</v>
       </c>
-      <c r="R5" s="9" t="n">
+      <c r="R5" s="15" t="n">
         <v>165</v>
       </c>
-      <c r="S5" s="13" t="n">
+      <c r="S5" s="15" t="n">
         <f aca="false">(L5+M5)*N5/100*(1-O5)-K5-P5-Q5-R5</f>
         <v>2768.10606060605</v>
       </c>
-      <c r="T5" s="13" t="n">
+      <c r="T5" s="15" t="n">
         <f aca="false">ROUNDUP((K5+P5)*0.090909,0)</f>
         <v>2080</v>
       </c>
-      <c r="U5" s="13" t="n">
+      <c r="U5" s="15" t="n">
         <f aca="false">S5+T5</f>
         <v>4848.10606060605</v>
       </c>
-      <c r="V5" s="14" t="n">
+      <c r="V5" s="16" t="n">
         <v>0.12</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="n">
-        <v>4</v>
+        <v>271</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>23</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="F6" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="G6" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="H6" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="G6" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="J6" s="8" t="n">
+      <c r="I6" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="J6" s="9" t="n">
         <v>0.75</v>
       </c>
-      <c r="K6" s="9" t="n">
+      <c r="K6" s="10" t="n">
         <v>11900</v>
       </c>
-      <c r="L6" s="10" t="n">
+      <c r="L6" s="11" t="n">
         <f aca="false">(K6+P6+Q6+R6-K6/11)/(1-V6-O6)/N6*100</f>
-        <v>3065.30583613917</v>
-      </c>
-      <c r="M6" s="11" t="n">
+        <v>2903.97395002658</v>
+      </c>
+      <c r="M6" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="N6" s="8" t="n">
-        <v>900</v>
-      </c>
-      <c r="O6" s="12" t="n">
+      <c r="N6" s="13" t="n">
+        <v>950</v>
+      </c>
+      <c r="O6" s="14" t="n">
         <v>0.16</v>
       </c>
-      <c r="P6" s="9" t="n">
+      <c r="P6" s="10" t="n">
         <v>2080</v>
       </c>
-      <c r="Q6" s="13" t="n">
+      <c r="Q6" s="15" t="n">
         <f aca="false">VLOOKUP(J6,kse요율!$A$4:$C$28,3,0)</f>
         <v>6800</v>
       </c>
-      <c r="R6" s="9" t="n">
+      <c r="R6" s="15" t="n">
         <v>165</v>
       </c>
-      <c r="S6" s="13" t="n">
+      <c r="S6" s="15" t="n">
         <f aca="false">(L6+M6)*N6/100*(1-O6)-K6-P6-Q6-R6</f>
         <v>2228.71212121212</v>
       </c>
-      <c r="T6" s="13" t="n">
+      <c r="T6" s="15" t="n">
         <f aca="false">ROUNDUP((K6+P6)*0.090909,0)</f>
         <v>1271</v>
       </c>
-      <c r="U6" s="13" t="n">
+      <c r="U6" s="15" t="n">
         <f aca="false">S6+T6</f>
         <v>3499.71212121212</v>
       </c>
-      <c r="V6" s="14" t="n">
+      <c r="V6" s="16" t="n">
         <v>0.12</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="n">
-        <v>5</v>
+        <v>272</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>23</v>
       </c>
       <c r="C7" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F7" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="G7" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="H7" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="F7" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="J7" s="8" t="n">
+      <c r="I7" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="J7" s="9" t="n">
         <v>0.75</v>
       </c>
-      <c r="K7" s="9" t="n">
+      <c r="K7" s="10" t="n">
         <v>12110</v>
       </c>
-      <c r="L7" s="10" t="n">
+      <c r="L7" s="11" t="n">
         <f aca="false">(K7+P7+Q7+R7-K7/11)/(1-V7-O7)/N7*100</f>
-        <v>3094.76711560045</v>
-      </c>
-      <c r="M7" s="11" t="n">
+        <v>2931.884635832</v>
+      </c>
+      <c r="M7" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="N7" s="8" t="n">
-        <v>900</v>
-      </c>
-      <c r="O7" s="12" t="n">
+      <c r="N7" s="13" t="n">
+        <v>950</v>
+      </c>
+      <c r="O7" s="14" t="n">
         <v>0.16</v>
       </c>
-      <c r="P7" s="9" t="n">
+      <c r="P7" s="10" t="n">
         <v>2080</v>
       </c>
-      <c r="Q7" s="13" t="n">
+      <c r="Q7" s="15" t="n">
         <f aca="false">VLOOKUP(J7,kse요율!$A$4:$C$28,3,0)</f>
         <v>6800</v>
       </c>
-      <c r="R7" s="9" t="n">
+      <c r="R7" s="15" t="n">
         <v>165</v>
       </c>
-      <c r="S7" s="13" t="n">
+      <c r="S7" s="15" t="n">
         <f aca="false">(L7+M7)*N7/100*(1-O7)-K7-P7-Q7-R7</f>
         <v>2241.4393939394</v>
       </c>
-      <c r="T7" s="13" t="n">
+      <c r="T7" s="15" t="n">
         <f aca="false">ROUNDUP((K7+P7)*0.090909,0)</f>
         <v>1290</v>
       </c>
-      <c r="U7" s="13" t="n">
+      <c r="U7" s="15" t="n">
         <f aca="false">S7+T7</f>
         <v>3531.4393939394</v>
       </c>
-      <c r="V7" s="14" t="n">
+      <c r="V7" s="16" t="n">
         <v>0.12</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="n">
-        <v>6</v>
+        <v>273</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>23</v>
       </c>
       <c r="C8" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="G8" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="H8" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="E8" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="J8" s="8" t="n">
+      <c r="I8" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="J8" s="9" t="n">
         <v>0.75</v>
       </c>
-      <c r="K8" s="9" t="n">
+      <c r="K8" s="10" t="n">
         <v>13000</v>
       </c>
-      <c r="L8" s="10" t="n">
+      <c r="L8" s="11" t="n">
         <f aca="false">(K8+P8+Q8+R8-K8/11)/(1-V8-O8)/N8*100</f>
-        <v>3219.62682379349</v>
-      </c>
-      <c r="M8" s="11" t="n">
+        <v>3050.17278043594</v>
+      </c>
+      <c r="M8" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="N8" s="8" t="n">
-        <v>900</v>
-      </c>
-      <c r="O8" s="12" t="n">
+      <c r="N8" s="13" t="n">
+        <v>950</v>
+      </c>
+      <c r="O8" s="14" t="n">
         <v>0.16</v>
       </c>
-      <c r="P8" s="9" t="n">
+      <c r="P8" s="10" t="n">
         <v>2080</v>
       </c>
-      <c r="Q8" s="13" t="n">
+      <c r="Q8" s="15" t="n">
         <f aca="false">VLOOKUP(J8,kse요율!$A$4:$C$28,3,0)</f>
         <v>6800</v>
       </c>
-      <c r="R8" s="9" t="n">
+      <c r="R8" s="15" t="n">
         <v>165</v>
       </c>
-      <c r="S8" s="13" t="n">
+      <c r="S8" s="15" t="n">
         <f aca="false">(L8+M8)*N8/100*(1-O8)-K8-P8-Q8-R8</f>
         <v>2295.37878787879</v>
       </c>
-      <c r="T8" s="13" t="n">
+      <c r="T8" s="15" t="n">
         <f aca="false">ROUNDUP((K8+P8)*0.090909,0)</f>
         <v>1371</v>
       </c>
-      <c r="U8" s="13" t="n">
+      <c r="U8" s="15" t="n">
         <f aca="false">S8+T8</f>
         <v>3666.37878787879</v>
       </c>
-      <c r="V8" s="14" t="n">
+      <c r="V8" s="16" t="n">
         <v>0.12</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="n">
-        <v>7</v>
+        <v>274</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>23</v>
       </c>
       <c r="C9" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="H9" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="J9" s="8" t="n">
+      <c r="I9" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="J9" s="9" t="n">
         <v>0.75</v>
       </c>
-      <c r="K9" s="9" t="n">
+      <c r="K9" s="10" t="n">
         <v>29000</v>
       </c>
-      <c r="L9" s="10" t="n">
+      <c r="L9" s="11" t="n">
         <f aca="false">(K9+P9+Q9+R9-K9/11)/(1-V9-O9)/N9*100</f>
-        <v>5464.29573512907</v>
-      </c>
-      <c r="M9" s="11" t="n">
+        <v>5176.70122275385</v>
+      </c>
+      <c r="M9" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="N9" s="8" t="n">
-        <v>900</v>
-      </c>
-      <c r="O9" s="12" t="n">
+      <c r="N9" s="13" t="n">
+        <v>950</v>
+      </c>
+      <c r="O9" s="14" t="n">
         <v>0.16</v>
       </c>
-      <c r="P9" s="9" t="n">
+      <c r="P9" s="10" t="n">
         <v>2080</v>
       </c>
-      <c r="Q9" s="13" t="n">
+      <c r="Q9" s="15" t="n">
         <f aca="false">VLOOKUP(J9,kse요율!$A$4:$C$28,3,0)</f>
         <v>6800</v>
       </c>
-      <c r="R9" s="9" t="n">
+      <c r="R9" s="15" t="n">
         <v>165</v>
       </c>
-      <c r="S9" s="13" t="n">
+      <c r="S9" s="15" t="n">
         <f aca="false">(L9+M9)*N9/100*(1-O9)-K9-P9-Q9-R9</f>
         <v>3265.07575757575</v>
       </c>
-      <c r="T9" s="13" t="n">
+      <c r="T9" s="15" t="n">
         <f aca="false">ROUNDUP((K9+P9)*0.090909,0)</f>
         <v>2826</v>
       </c>
-      <c r="U9" s="13" t="n">
+      <c r="U9" s="15" t="n">
         <f aca="false">S9+T9</f>
         <v>6091.07575757575</v>
       </c>
-      <c r="V9" s="14" t="n">
+      <c r="V9" s="16" t="n">
         <v>0.12</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="16" t="s">
-        <v>74</v>
-      </c>
-    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="I3" r:id="rId1" display="바로가기"/>
+    <hyperlink ref="I4" r:id="rId2" display="바로가기"/>
+    <hyperlink ref="I5" r:id="rId3" display="바로가기"/>
+    <hyperlink ref="I6" r:id="rId4" display="바로가기"/>
+    <hyperlink ref="I7" r:id="rId5" display="바로가기"/>
+    <hyperlink ref="I8" r:id="rId6" display="바로가기"/>
+    <hyperlink ref="I9" r:id="rId7" display="바로가기"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2427,7 +2125,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2435,10 +2133,10 @@
         <v>10</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Margin calculator v2: MSRP (정가) instead of sale price, weight=2x content estimate rounded to tier, sources restricted to official malls/musinsa only
</commit_message>
<xml_diff>
--- a/data/마진계산기_템플릿.xlsx
+++ b/data/마진계산기_템플릿.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="72">
   <si>
     <r>
       <rPr>
@@ -124,8 +124,49 @@
     <t xml:space="preserve">무게</t>
   </si>
   <si>
-    <t xml:space="preserve">국내
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">국내
 구매가</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">정가</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">큐텐 판매가</t>
@@ -864,6 +905,219 @@
   </si>
   <si>
     <t xml:space="preserve">올인원</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">※ 무게는 실제 제품 내용물 추정 무게 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">× 2(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">포장 감안</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">를 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">kse</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">요율표 구간에 올림 적용한 값입니다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">실측 아님</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확인 후 수정 권장</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">※ 국내구매가는 각 공식몰</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">무신사에 표시된 소비자가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">정가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">기준입니다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">세일 종료 시 변동될 수 있습니다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
   </si>
   <si>
     <r>
@@ -1011,7 +1265,7 @@
     <numFmt numFmtId="171" formatCode="\₩#,##0"/>
     <numFmt numFmtId="172" formatCode="0.00%"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1072,6 +1326,19 @@
       <color rgb="FF0563C1"/>
       <name val="Noto Sans CJK SC"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF666666"/>
+      <name val="Noto Sans CJK SC"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF666666"/>
+      <name val="맑은 고딕"/>
+      <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -1155,7 +1422,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1232,6 +1499,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1289,7 +1560,7 @@
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF666666"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
@@ -1484,7 +1755,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:V9"/>
+  <dimension ref="A1:V13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5.38"/>
@@ -1580,7 +1851,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="n">
         <v>268</v>
       </c>
@@ -1609,14 +1880,14 @@
         <v>30</v>
       </c>
       <c r="J3" s="9" t="n">
-        <v>0.75</v>
+        <v>0.25</v>
       </c>
       <c r="K3" s="10" t="n">
-        <v>17600</v>
+        <v>20000</v>
       </c>
       <c r="L3" s="11" t="n">
         <f aca="false">(K3+P3+Q3+R3-K3/11)/(1-V3-O3)/N3*100</f>
-        <v>3661.54970760234</v>
+        <v>3753.92078681552</v>
       </c>
       <c r="M3" s="12" t="n">
         <v>0</v>
@@ -1632,28 +1903,28 @@
       </c>
       <c r="Q3" s="15" t="n">
         <f aca="false">VLOOKUP(J3,kse요율!$A$4:$C$28,3,0)</f>
-        <v>6800</v>
+        <v>5250</v>
       </c>
       <c r="R3" s="15" t="n">
         <v>165</v>
       </c>
       <c r="S3" s="15" t="n">
         <f aca="false">(L3+M3)*N3/100*(1-O3)-K3-P3-Q3-R3</f>
-        <v>2574.16666666667</v>
+        <v>2461.28787878787</v>
       </c>
       <c r="T3" s="15" t="n">
         <f aca="false">ROUNDUP((K3+P3)*0.090909,0)</f>
-        <v>1790</v>
+        <v>2008</v>
       </c>
       <c r="U3" s="15" t="n">
         <f aca="false">S3+T3</f>
-        <v>4364.16666666667</v>
+        <v>4469.28787878787</v>
       </c>
       <c r="V3" s="16" t="n">
         <v>0.12</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="n">
         <v>269</v>
       </c>
@@ -1682,14 +1953,14 @@
         <v>30</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="K4" s="10" t="n">
-        <v>12900</v>
+        <v>32000</v>
       </c>
       <c r="L4" s="11" t="n">
         <f aca="false">(K4+P4+Q4+R4-K4/11)/(1-V4-O4)/N4*100</f>
-        <v>2905.30303030303</v>
+        <v>5348.81711855396</v>
       </c>
       <c r="M4" s="12" t="n">
         <v>0</v>
@@ -1705,28 +1976,28 @@
       </c>
       <c r="Q4" s="15" t="n">
         <f aca="false">VLOOKUP(J4,kse요율!$A$4:$C$28,3,0)</f>
-        <v>5900</v>
+        <v>5250</v>
       </c>
       <c r="R4" s="15" t="n">
         <v>165</v>
       </c>
       <c r="S4" s="15" t="n">
         <f aca="false">(L4+M4)*N4/100*(1-O4)-K4-P4-Q4-R4</f>
-        <v>2139.31818181819</v>
+        <v>3188.56060606059</v>
       </c>
       <c r="T4" s="15" t="n">
         <f aca="false">ROUNDUP((K4+P4)*0.090909,0)</f>
-        <v>1362</v>
+        <v>3099</v>
       </c>
       <c r="U4" s="15" t="n">
         <f aca="false">S4+T4</f>
-        <v>3501.31818181819</v>
+        <v>6287.56060606059</v>
       </c>
       <c r="V4" s="16" t="n">
         <v>0.12</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="n">
         <v>270</v>
       </c>
@@ -1799,7 +2070,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="n">
         <v>271</v>
       </c>
@@ -1828,14 +2099,14 @@
         <v>30</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="K6" s="10" t="n">
-        <v>11900</v>
+        <v>13000</v>
       </c>
       <c r="L6" s="11" t="n">
         <f aca="false">(K6+P6+Q6+R6-K6/11)/(1-V6-O6)/N6*100</f>
-        <v>2903.97395002658</v>
+        <v>2918.59383306752</v>
       </c>
       <c r="M6" s="12" t="n">
         <v>0</v>
@@ -1851,28 +2122,28 @@
       </c>
       <c r="Q6" s="15" t="n">
         <f aca="false">VLOOKUP(J6,kse요율!$A$4:$C$28,3,0)</f>
-        <v>6800</v>
+        <v>5900</v>
       </c>
       <c r="R6" s="15" t="n">
         <v>165</v>
       </c>
       <c r="S6" s="15" t="n">
         <f aca="false">(L6+M6)*N6/100*(1-O6)-K6-P6-Q6-R6</f>
-        <v>2228.71212121212</v>
+        <v>2145.37878787879</v>
       </c>
       <c r="T6" s="15" t="n">
         <f aca="false">ROUNDUP((K6+P6)*0.090909,0)</f>
-        <v>1271</v>
+        <v>1371</v>
       </c>
       <c r="U6" s="15" t="n">
         <f aca="false">S6+T6</f>
-        <v>3499.71212121212</v>
+        <v>3516.37878787879</v>
       </c>
       <c r="V6" s="16" t="n">
         <v>0.12</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="n">
         <v>272</v>
       </c>
@@ -1901,14 +2172,14 @@
         <v>30</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="K7" s="10" t="n">
-        <v>12110</v>
+        <v>19900</v>
       </c>
       <c r="L7" s="11" t="n">
         <f aca="false">(K7+P7+Q7+R7-K7/11)/(1-V7-O7)/N7*100</f>
-        <v>2931.884635832</v>
+        <v>3835.65922381712</v>
       </c>
       <c r="M7" s="12" t="n">
         <v>0</v>
@@ -1924,28 +2195,28 @@
       </c>
       <c r="Q7" s="15" t="n">
         <f aca="false">VLOOKUP(J7,kse요율!$A$4:$C$28,3,0)</f>
-        <v>6800</v>
+        <v>5900</v>
       </c>
       <c r="R7" s="15" t="n">
         <v>165</v>
       </c>
       <c r="S7" s="15" t="n">
         <f aca="false">(L7+M7)*N7/100*(1-O7)-K7-P7-Q7-R7</f>
-        <v>2241.4393939394</v>
+        <v>2563.56060606061</v>
       </c>
       <c r="T7" s="15" t="n">
         <f aca="false">ROUNDUP((K7+P7)*0.090909,0)</f>
-        <v>1290</v>
+        <v>1999</v>
       </c>
       <c r="U7" s="15" t="n">
         <f aca="false">S7+T7</f>
-        <v>3531.4393939394</v>
+        <v>4562.56060606061</v>
       </c>
       <c r="V7" s="16" t="n">
         <v>0.12</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="n">
         <v>273</v>
       </c>
@@ -1974,14 +2245,14 @@
         <v>30</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>0.75</v>
+        <v>0.25</v>
       </c>
       <c r="K8" s="10" t="n">
-        <v>13000</v>
+        <v>20000</v>
       </c>
       <c r="L8" s="11" t="n">
         <f aca="false">(K8+P8+Q8+R8-K8/11)/(1-V8-O8)/N8*100</f>
-        <v>3050.17278043594</v>
+        <v>3753.92078681552</v>
       </c>
       <c r="M8" s="12" t="n">
         <v>0</v>
@@ -1997,28 +2268,28 @@
       </c>
       <c r="Q8" s="15" t="n">
         <f aca="false">VLOOKUP(J8,kse요율!$A$4:$C$28,3,0)</f>
-        <v>6800</v>
+        <v>5250</v>
       </c>
       <c r="R8" s="15" t="n">
         <v>165</v>
       </c>
       <c r="S8" s="15" t="n">
         <f aca="false">(L8+M8)*N8/100*(1-O8)-K8-P8-Q8-R8</f>
-        <v>2295.37878787879</v>
+        <v>2461.28787878787</v>
       </c>
       <c r="T8" s="15" t="n">
         <f aca="false">ROUNDUP((K8+P8)*0.090909,0)</f>
-        <v>1371</v>
+        <v>2008</v>
       </c>
       <c r="U8" s="15" t="n">
         <f aca="false">S8+T8</f>
-        <v>3666.37878787879</v>
+        <v>4469.28787878787</v>
       </c>
       <c r="V8" s="16" t="n">
         <v>0.12</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="n">
         <v>274</v>
       </c>
@@ -2047,14 +2318,14 @@
         <v>30</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>0.75</v>
+        <v>0.1</v>
       </c>
       <c r="K9" s="10" t="n">
-        <v>29000</v>
+        <v>50000</v>
       </c>
       <c r="L9" s="11" t="n">
         <f aca="false">(K9+P9+Q9+R9-K9/11)/(1-V9-O9)/N9*100</f>
-        <v>5176.70122275385</v>
+        <v>7631.5124933546</v>
       </c>
       <c r="M9" s="12" t="n">
         <v>0</v>
@@ -2070,25 +2341,35 @@
       </c>
       <c r="Q9" s="15" t="n">
         <f aca="false">VLOOKUP(J9,kse요율!$A$4:$C$28,3,0)</f>
-        <v>6800</v>
+        <v>4500</v>
       </c>
       <c r="R9" s="15" t="n">
         <v>165</v>
       </c>
       <c r="S9" s="15" t="n">
         <f aca="false">(L9+M9)*N9/100*(1-O9)-K9-P9-Q9-R9</f>
-        <v>3265.07575757575</v>
+        <v>4154.4696969697</v>
       </c>
       <c r="T9" s="15" t="n">
         <f aca="false">ROUNDUP((K9+P9)*0.090909,0)</f>
-        <v>2826</v>
+        <v>4735</v>
       </c>
       <c r="U9" s="15" t="n">
         <f aca="false">S9+T9</f>
-        <v>6091.07575757575</v>
+        <v>8889.4696969697</v>
       </c>
       <c r="V9" s="16" t="n">
         <v>0.12</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="17" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="17" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -2124,19 +2405,19 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
-        <v>67</v>
+      <c r="A1" s="18" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="18" t="s">
-        <v>68</v>
-      </c>
-      <c r="C3" s="18" t="s">
-        <v>69</v>
+      <c r="B3" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Fix weight logic: base kse tier + 2 tier-steps up (not doubling)
</commit_message>
<xml_diff>
--- a/data/마진계산기_템플릿.xlsx
+++ b/data/마진계산기_템플릿.xlsx
@@ -464,7 +464,7 @@
     <t xml:space="preserve">올인원</t>
   </si>
   <si>
-    <t xml:space="preserve">※ 무게는 실제 제품 내용물 추정 무게 × 2(포장 감안)를 kse요율표 구간에 올림 적용한 값입니다. 실측 아님, 확인 후 수정 권장.</t>
+    <t xml:space="preserve">※ 무게는 실제 제품 내용물 추정치를 kse요율표 구간으로 올림한 뒤, 거기서 2단계 더 올린 값입니다(포장·박스 감안 버퍼). 실측 아님, 확인 후 수정 권장.</t>
   </si>
   <si>
     <t xml:space="preserve">※ 국내구매가는 각 공식몰/무신사에 표시된 소비자가(정가) 기준입니다. 세일 종료 시 변동될 수 있습니다.</t>
@@ -1157,14 +1157,14 @@
         <v>30</v>
       </c>
       <c r="J3" s="10" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="K3" s="11" t="n">
         <v>20000</v>
       </c>
       <c r="L3" s="12" t="n">
         <f aca="false">(K3+P3+Q3+R3-K3/11)/(1-V3-O3)/N3*100</f>
-        <v>3753.92078681552</v>
+        <v>3848.95002658161</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>0</v>
@@ -1180,14 +1180,14 @@
       </c>
       <c r="Q3" s="16" t="n">
         <f aca="false">VLOOKUP(J3,kse요율!$A$4:$C$28,3,0)</f>
-        <v>5250</v>
+        <v>5900</v>
       </c>
       <c r="R3" s="16" t="n">
         <v>165</v>
       </c>
       <c r="S3" s="16" t="n">
         <f aca="false">(L3+M3)*N3/100*(1-O3)-K3-P3-Q3-R3</f>
-        <v>2461.28787878787</v>
+        <v>2569.62121212121</v>
       </c>
       <c r="T3" s="16" t="n">
         <f aca="false">ROUNDUP((K3+P3)*0.090909,0)</f>
@@ -1195,7 +1195,7 @@
       </c>
       <c r="U3" s="16" t="n">
         <f aca="false">S3+T3</f>
-        <v>4469.28787878787</v>
+        <v>4577.62121212121</v>
       </c>
       <c r="V3" s="17" t="n">
         <v>0.12</v>
@@ -1230,14 +1230,14 @@
         <v>30</v>
       </c>
       <c r="J4" s="10" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="K4" s="11" t="n">
         <v>32000</v>
       </c>
       <c r="L4" s="12" t="n">
         <f aca="false">(K4+P4+Q4+R4-K4/11)/(1-V4-O4)/N4*100</f>
-        <v>5348.81711855396</v>
+        <v>5443.84635832004</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>0</v>
@@ -1253,14 +1253,14 @@
       </c>
       <c r="Q4" s="16" t="n">
         <f aca="false">VLOOKUP(J4,kse요율!$A$4:$C$28,3,0)</f>
-        <v>5250</v>
+        <v>5900</v>
       </c>
       <c r="R4" s="16" t="n">
         <v>165</v>
       </c>
       <c r="S4" s="16" t="n">
         <f aca="false">(L4+M4)*N4/100*(1-O4)-K4-P4-Q4-R4</f>
-        <v>3188.56060606059</v>
+        <v>3296.89393939394</v>
       </c>
       <c r="T4" s="16" t="n">
         <f aca="false">ROUNDUP((K4+P4)*0.090909,0)</f>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="U4" s="16" t="n">
         <f aca="false">S4+T4</f>
-        <v>6287.56060606059</v>
+        <v>6395.89393939394</v>
       </c>
       <c r="V4" s="17" t="n">
         <v>0.12</v>
@@ -1303,14 +1303,14 @@
         <v>30</v>
       </c>
       <c r="J5" s="10" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="K5" s="11" t="n">
         <v>20800</v>
       </c>
       <c r="L5" s="12" t="n">
         <f aca="false">(K5+P5+Q5+R5-K5/11)/(1-V5-O5)/N5*100</f>
-        <v>4086.85539606592</v>
+        <v>4145.33492822967</v>
       </c>
       <c r="M5" s="13" t="n">
         <v>0</v>
@@ -1326,14 +1326,14 @@
       </c>
       <c r="Q5" s="16" t="n">
         <f aca="false">VLOOKUP(J5,kse요율!$A$4:$C$28,3,0)</f>
-        <v>6800</v>
+        <v>7200</v>
       </c>
       <c r="R5" s="16" t="n">
         <v>165</v>
       </c>
       <c r="S5" s="16" t="n">
         <f aca="false">(L5+M5)*N5/100*(1-O5)-K5-P5-Q5-R5</f>
-        <v>2768.10606060605</v>
+        <v>2834.77272727273</v>
       </c>
       <c r="T5" s="16" t="n">
         <f aca="false">ROUNDUP((K5+P5)*0.090909,0)</f>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="U5" s="16" t="n">
         <f aca="false">S5+T5</f>
-        <v>4848.10606060605</v>
+        <v>4914.77272727273</v>
       </c>
       <c r="V5" s="17" t="n">
         <v>0.12</v>
@@ -1376,14 +1376,14 @@
         <v>30</v>
       </c>
       <c r="J6" s="10" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="K6" s="11" t="n">
         <v>13000</v>
       </c>
       <c r="L6" s="12" t="n">
         <f aca="false">(K6+P6+Q6+R6-K6/11)/(1-V6-O6)/N6*100</f>
-        <v>2918.59383306752</v>
+        <v>3050.17278043594</v>
       </c>
       <c r="M6" s="13" t="n">
         <v>0</v>
@@ -1399,14 +1399,14 @@
       </c>
       <c r="Q6" s="16" t="n">
         <f aca="false">VLOOKUP(J6,kse요율!$A$4:$C$28,3,0)</f>
-        <v>5900</v>
+        <v>6800</v>
       </c>
       <c r="R6" s="16" t="n">
         <v>165</v>
       </c>
       <c r="S6" s="16" t="n">
         <f aca="false">(L6+M6)*N6/100*(1-O6)-K6-P6-Q6-R6</f>
-        <v>2145.37878787879</v>
+        <v>2295.37878787879</v>
       </c>
       <c r="T6" s="16" t="n">
         <f aca="false">ROUNDUP((K6+P6)*0.090909,0)</f>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="U6" s="16" t="n">
         <f aca="false">S6+T6</f>
-        <v>3516.37878787879</v>
+        <v>3666.37878787879</v>
       </c>
       <c r="V6" s="17" t="n">
         <v>0.12</v>
@@ -1449,14 +1449,14 @@
         <v>30</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="K7" s="11" t="n">
         <v>19900</v>
       </c>
       <c r="L7" s="12" t="n">
         <f aca="false">(K7+P7+Q7+R7-K7/11)/(1-V7-O7)/N7*100</f>
-        <v>3835.65922381712</v>
+        <v>3967.23817118554</v>
       </c>
       <c r="M7" s="13" t="n">
         <v>0</v>
@@ -1472,14 +1472,14 @@
       </c>
       <c r="Q7" s="16" t="n">
         <f aca="false">VLOOKUP(J7,kse요율!$A$4:$C$28,3,0)</f>
-        <v>5900</v>
+        <v>6800</v>
       </c>
       <c r="R7" s="16" t="n">
         <v>165</v>
       </c>
       <c r="S7" s="16" t="n">
         <f aca="false">(L7+M7)*N7/100*(1-O7)-K7-P7-Q7-R7</f>
-        <v>2563.56060606061</v>
+        <v>2713.56060606061</v>
       </c>
       <c r="T7" s="16" t="n">
         <f aca="false">ROUNDUP((K7+P7)*0.090909,0)</f>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="U7" s="16" t="n">
         <f aca="false">S7+T7</f>
-        <v>4562.56060606061</v>
+        <v>4712.56060606061</v>
       </c>
       <c r="V7" s="17" t="n">
         <v>0.12</v>
@@ -1522,14 +1522,14 @@
         <v>30</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="K8" s="11" t="n">
         <v>20000</v>
       </c>
       <c r="L8" s="12" t="n">
         <f aca="false">(K8+P8+Q8+R8-K8/11)/(1-V8-O8)/N8*100</f>
-        <v>3753.92078681552</v>
+        <v>3848.95002658161</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>0</v>
@@ -1545,14 +1545,14 @@
       </c>
       <c r="Q8" s="16" t="n">
         <f aca="false">VLOOKUP(J8,kse요율!$A$4:$C$28,3,0)</f>
-        <v>5250</v>
+        <v>5900</v>
       </c>
       <c r="R8" s="16" t="n">
         <v>165</v>
       </c>
       <c r="S8" s="16" t="n">
         <f aca="false">(L8+M8)*N8/100*(1-O8)-K8-P8-Q8-R8</f>
-        <v>2461.28787878787</v>
+        <v>2569.62121212121</v>
       </c>
       <c r="T8" s="16" t="n">
         <f aca="false">ROUNDUP((K8+P8)*0.090909,0)</f>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="U8" s="16" t="n">
         <f aca="false">S8+T8</f>
-        <v>4469.28787878787</v>
+        <v>4577.62121212121</v>
       </c>
       <c r="V8" s="17" t="n">
         <v>0.12</v>
@@ -1595,14 +1595,14 @@
         <v>30</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="K9" s="11" t="n">
         <v>50000</v>
       </c>
       <c r="L9" s="12" t="n">
         <f aca="false">(K9+P9+Q9+R9-K9/11)/(1-V9-O9)/N9*100</f>
-        <v>7631.5124933546</v>
+        <v>7836.1908559277</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>0</v>
@@ -1618,14 +1618,14 @@
       </c>
       <c r="Q9" s="16" t="n">
         <f aca="false">VLOOKUP(J9,kse요율!$A$4:$C$28,3,0)</f>
-        <v>4500</v>
+        <v>5900</v>
       </c>
       <c r="R9" s="16" t="n">
         <v>165</v>
       </c>
       <c r="S9" s="16" t="n">
         <f aca="false">(L9+M9)*N9/100*(1-O9)-K9-P9-Q9-R9</f>
-        <v>4154.4696969697</v>
+        <v>4387.80303030303</v>
       </c>
       <c r="T9" s="16" t="n">
         <f aca="false">ROUNDUP((K9+P9)*0.090909,0)</f>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="U9" s="16" t="n">
         <f aca="false">S9+T9</f>
-        <v>8889.4696969697</v>
+        <v>9122.80303030303</v>
       </c>
       <c r="V9" s="17" t="n">
         <v>0.12</v>

</xml_diff>

<commit_message>
Apply 0.75kg minimum weight floor
</commit_message>
<xml_diff>
--- a/data/마진계산기_템플릿.xlsx
+++ b/data/마진계산기_템플릿.xlsx
@@ -464,7 +464,7 @@
     <t xml:space="preserve">올인원</t>
   </si>
   <si>
-    <t xml:space="preserve">※ 무게는 실제 제품 내용물 추정치를 kse요율표 구간으로 올림한 뒤, 거기서 2단계 더 올린 값입니다(포장·박스 감안 버퍼). 실측 아님, 확인 후 수정 권장.</t>
+    <t xml:space="preserve">※ 무게는 실제 제품 내용물 추정치를 kse요율표 구간으로 올림한 뒤 2단계 더 올리고, 최소 0.75kg을 적용한 값입니다. 실측 아님, 확인 후 수정 권장.</t>
   </si>
   <si>
     <t xml:space="preserve">※ 국내구매가는 각 공식몰/무신사에 표시된 소비자가(정가) 기준입니다. 세일 종료 시 변동될 수 있습니다.</t>
@@ -1157,14 +1157,14 @@
         <v>30</v>
       </c>
       <c r="J3" s="10" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="K3" s="11" t="n">
         <v>20000</v>
       </c>
       <c r="L3" s="12" t="n">
         <f aca="false">(K3+P3+Q3+R3-K3/11)/(1-V3-O3)/N3*100</f>
-        <v>3848.95002658161</v>
+        <v>3980.52897395003</v>
       </c>
       <c r="M3" s="13" t="n">
         <v>0</v>
@@ -1180,14 +1180,14 @@
       </c>
       <c r="Q3" s="16" t="n">
         <f aca="false">VLOOKUP(J3,kse요율!$A$4:$C$28,3,0)</f>
-        <v>5900</v>
+        <v>6800</v>
       </c>
       <c r="R3" s="16" t="n">
         <v>165</v>
       </c>
       <c r="S3" s="16" t="n">
         <f aca="false">(L3+M3)*N3/100*(1-O3)-K3-P3-Q3-R3</f>
-        <v>2569.62121212121</v>
+        <v>2719.62121212121</v>
       </c>
       <c r="T3" s="16" t="n">
         <f aca="false">ROUNDUP((K3+P3)*0.090909,0)</f>
@@ -1195,7 +1195,7 @@
       </c>
       <c r="U3" s="16" t="n">
         <f aca="false">S3+T3</f>
-        <v>4577.62121212121</v>
+        <v>4727.62121212121</v>
       </c>
       <c r="V3" s="17" t="n">
         <v>0.12</v>
@@ -1230,14 +1230,14 @@
         <v>30</v>
       </c>
       <c r="J4" s="10" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="K4" s="11" t="n">
         <v>32000</v>
       </c>
       <c r="L4" s="12" t="n">
         <f aca="false">(K4+P4+Q4+R4-K4/11)/(1-V4-O4)/N4*100</f>
-        <v>5443.84635832004</v>
+        <v>5575.42530568846</v>
       </c>
       <c r="M4" s="13" t="n">
         <v>0</v>
@@ -1253,14 +1253,14 @@
       </c>
       <c r="Q4" s="16" t="n">
         <f aca="false">VLOOKUP(J4,kse요율!$A$4:$C$28,3,0)</f>
-        <v>5900</v>
+        <v>6800</v>
       </c>
       <c r="R4" s="16" t="n">
         <v>165</v>
       </c>
       <c r="S4" s="16" t="n">
         <f aca="false">(L4+M4)*N4/100*(1-O4)-K4-P4-Q4-R4</f>
-        <v>3296.89393939394</v>
+        <v>3446.89393939394</v>
       </c>
       <c r="T4" s="16" t="n">
         <f aca="false">ROUNDUP((K4+P4)*0.090909,0)</f>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="U4" s="16" t="n">
         <f aca="false">S4+T4</f>
-        <v>6395.89393939394</v>
+        <v>6545.89393939394</v>
       </c>
       <c r="V4" s="17" t="n">
         <v>0.12</v>
@@ -1522,14 +1522,14 @@
         <v>30</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="K8" s="11" t="n">
         <v>20000</v>
       </c>
       <c r="L8" s="12" t="n">
         <f aca="false">(K8+P8+Q8+R8-K8/11)/(1-V8-O8)/N8*100</f>
-        <v>3848.95002658161</v>
+        <v>3980.52897395003</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>0</v>
@@ -1545,14 +1545,14 @@
       </c>
       <c r="Q8" s="16" t="n">
         <f aca="false">VLOOKUP(J8,kse요율!$A$4:$C$28,3,0)</f>
-        <v>5900</v>
+        <v>6800</v>
       </c>
       <c r="R8" s="16" t="n">
         <v>165</v>
       </c>
       <c r="S8" s="16" t="n">
         <f aca="false">(L8+M8)*N8/100*(1-O8)-K8-P8-Q8-R8</f>
-        <v>2569.62121212121</v>
+        <v>2719.62121212121</v>
       </c>
       <c r="T8" s="16" t="n">
         <f aca="false">ROUNDUP((K8+P8)*0.090909,0)</f>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="U8" s="16" t="n">
         <f aca="false">S8+T8</f>
-        <v>4577.62121212121</v>
+        <v>4727.62121212121</v>
       </c>
       <c r="V8" s="17" t="n">
         <v>0.12</v>
@@ -1595,14 +1595,14 @@
         <v>30</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="K9" s="11" t="n">
         <v>50000</v>
       </c>
       <c r="L9" s="12" t="n">
         <f aca="false">(K9+P9+Q9+R9-K9/11)/(1-V9-O9)/N9*100</f>
-        <v>7836.1908559277</v>
+        <v>7967.76980329612</v>
       </c>
       <c r="M9" s="13" t="n">
         <v>0</v>
@@ -1618,14 +1618,14 @@
       </c>
       <c r="Q9" s="16" t="n">
         <f aca="false">VLOOKUP(J9,kse요율!$A$4:$C$28,3,0)</f>
-        <v>5900</v>
+        <v>6800</v>
       </c>
       <c r="R9" s="16" t="n">
         <v>165</v>
       </c>
       <c r="S9" s="16" t="n">
         <f aca="false">(L9+M9)*N9/100*(1-O9)-K9-P9-Q9-R9</f>
-        <v>4387.80303030303</v>
+        <v>4537.80303030303</v>
       </c>
       <c r="T9" s="16" t="n">
         <f aca="false">ROUNDUP((K9+P9)*0.090909,0)</f>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="U9" s="16" t="n">
         <f aca="false">S9+T9</f>
-        <v>9122.80303030303</v>
+        <v>9272.80303030303</v>
       </c>
       <c r="V9" s="17" t="n">
         <v>0.12</v>

</xml_diff>

<commit_message>
Item name format: no. + brand + product name (Korean brand names for consistency)
</commit_message>
<xml_diff>
--- a/data/마진계산기_템플릿.xlsx
+++ b/data/마진계산기_템플릿.xlsx
@@ -139,7 +139,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">268. </t>
+      <t xml:space="preserve">268. celimax </t>
     </r>
     <r>
       <rPr>
@@ -188,7 +188,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">269. </t>
+      <t xml:space="preserve">269. Sung Boon Editor </t>
     </r>
     <r>
       <rPr>
@@ -224,7 +224,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">270. </t>
+      <t xml:space="preserve">270. GROWUS </t>
     </r>
     <r>
       <rPr>
@@ -279,7 +279,7 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">그린티 히알루론산 미스트 </t>
+      <t xml:space="preserve">이니스프리 그린티 히알루론산 미스트 </t>
     </r>
     <r>
       <rPr>
@@ -325,7 +325,7 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">단백질 본드 모이스트 앰플 에센스 </t>
+      <t xml:space="preserve">헤어플러스 단백질 본드 모이스트 앰플 에센스 </t>
     </r>
     <r>
       <rPr>
@@ -371,7 +371,7 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">닥터 마스크 시카 </t>
+      <t xml:space="preserve">로벡틴 닥터 마스크 시카 </t>
     </r>
     <r>
       <rPr>
@@ -417,7 +417,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">274. </t>
+      <t xml:space="preserve">274. KAHI </t>
     </r>
     <r>
       <rPr>

</xml_diff>

<commit_message>
Use Korean brand names consistently in item name column (celimax->셀리맥스 etc.)
</commit_message>
<xml_diff>
--- a/data/마진계산기_템플릿.xlsx
+++ b/data/마진계산기_템플릿.xlsx
@@ -139,7 +139,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">268. celimax </t>
+      <t xml:space="preserve">268. </t>
     </r>
     <r>
       <rPr>
@@ -148,7 +148,7 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">하트 핑크 톤업 선크림 </t>
+      <t xml:space="preserve">셀리맥스 하트 핑크 톤업 선크림 </t>
     </r>
     <r>
       <rPr>
@@ -188,7 +188,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">269. Sung Boon Editor </t>
+      <t xml:space="preserve">269. </t>
     </r>
     <r>
       <rPr>
@@ -197,7 +197,7 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">그린토마토 딥포어 클린 엔자임 파우더워시</t>
+      <t xml:space="preserve">성분에디터 그린토마토 딥포어 클린 엔자임 파우더워시</t>
     </r>
   </si>
   <si>
@@ -224,7 +224,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">270. GROWUS </t>
+      <t xml:space="preserve">270. </t>
     </r>
     <r>
       <rPr>
@@ -233,7 +233,7 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">데미지 테라피 노워시 트리트먼트 </t>
+      <t xml:space="preserve">그로우어스 데미지 테라피 노워시 트리트먼트 </t>
     </r>
     <r>
       <rPr>
@@ -417,7 +417,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">274. KAHI </t>
+      <t xml:space="preserve">274. </t>
     </r>
     <r>
       <rPr>
@@ -426,7 +426,7 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">멀티밤 리필키트 </t>
+      <t xml:space="preserve">가히 멀티밤 리필키트 </t>
     </r>
     <r>
       <rPr>

</xml_diff>

<commit_message>
Margin calculator: show actual URL text in source-link column instead of generic '바로가기'
</commit_message>
<xml_diff>
--- a/data/마진계산기_템플릿.xlsx
+++ b/data/마진계산기_템플릿.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="78">
   <si>
     <r>
       <rPr>
@@ -177,7 +177,7 @@
     <t xml:space="preserve">선크림・로션</t>
   </si>
   <si>
-    <t xml:space="preserve">바로가기</t>
+    <t xml:space="preserve">https://celimax.co.kr/product/하트핑크-톤업-선크림-40ml/54/</t>
   </si>
   <si>
     <r>
@@ -216,6 +216,9 @@
     <t xml:space="preserve">세안 파우더</t>
   </si>
   <si>
+    <t xml:space="preserve">https://sungboon.com/product/그린토마토-딥포어-클린-엔자임-파우더워시/517/category/262/display/1/</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -262,6 +265,9 @@
     <t xml:space="preserve">씻어내지 않는 트리트먼트</t>
   </si>
   <si>
+    <t xml:space="preserve">https://growus.kr/products/108131871</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -308,6 +314,9 @@
     <t xml:space="preserve">보습 미스트</t>
   </si>
   <si>
+    <t xml:space="preserve">https://www.musinsa.com/products/3229444</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -354,6 +363,9 @@
     <t xml:space="preserve">헤어 오일</t>
   </si>
   <si>
+    <t xml:space="preserve">https://www.hairplus.co.kr/goods/goods_view.php?goodsNo=1000000035</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -409,6 +421,9 @@
     <t xml:space="preserve">마스크 팩</t>
   </si>
   <si>
+    <t xml:space="preserve">https://rovectin.co.kr/product/트러블진정-닥터-마스크-시카-5매입/211/</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -462,6 +477,9 @@
   </si>
   <si>
     <t xml:space="preserve">올인원</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://kahicosmetics.co.kr/product/가히-멀티밤-리필키트-9g-x-2개/145</t>
   </si>
   <si>
     <t xml:space="preserve">※ 무게는 실제 제품 내용물 추정치를 kse요율표 구간으로 올림한 뒤 2단계 더 올리고, 최소 0.75kg을 적용한 값입니다. 실측 아님, 확인 후 수정 권장.</t>
@@ -1042,7 +1060,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="11.62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="6.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="12.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="11.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="11.38"/>
@@ -1227,7 +1245,7 @@
         <v>36</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="J4" s="10" t="n">
         <v>0.75</v>
@@ -1282,25 +1300,25 @@
         <v>23</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="J5" s="10" t="n">
         <v>1</v>
@@ -1355,25 +1373,25 @@
         <v>23</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>30</v>
+        <v>51</v>
       </c>
       <c r="J6" s="10" t="n">
         <v>0.75</v>
@@ -1428,25 +1446,25 @@
         <v>23</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="J7" s="10" t="n">
         <v>0.75</v>
@@ -1501,25 +1519,25 @@
         <v>23</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>30</v>
+        <v>65</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>0.75</v>
@@ -1574,25 +1592,25 @@
         <v>23</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>30</v>
+        <v>72</v>
       </c>
       <c r="J9" s="10" t="n">
         <v>0.75</v>
@@ -1641,23 +1659,23 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="I3" r:id="rId1" display="바로가기"/>
-    <hyperlink ref="I4" r:id="rId2" display="바로가기"/>
-    <hyperlink ref="I5" r:id="rId3" display="바로가기"/>
-    <hyperlink ref="I6" r:id="rId4" display="바로가기"/>
-    <hyperlink ref="I7" r:id="rId5" display="바로가기"/>
-    <hyperlink ref="I8" r:id="rId6" display="바로가기"/>
-    <hyperlink ref="I9" r:id="rId7" display="바로가기"/>
+    <hyperlink ref="I3" r:id="rId1" display="https://celimax.co.kr/product/하트핑크-톤업-선크림-40ml/54/"/>
+    <hyperlink ref="I4" r:id="rId2" display="https://sungboon.com/product/그린토마토-딥포어-클린-엔자임-파우더워시/517/category/262/display/1/"/>
+    <hyperlink ref="I5" r:id="rId3" display="https://growus.kr/products/108131871"/>
+    <hyperlink ref="I6" r:id="rId4" display="https://www.musinsa.com/products/3229444"/>
+    <hyperlink ref="I7" r:id="rId5" display="https://www.hairplus.co.kr/goods/goods_view.php?goodsNo=1000000035"/>
+    <hyperlink ref="I8" r:id="rId6" display="https://rovectin.co.kr/product/트러블진정-닥터-마스크-시카-5매입/211/"/>
+    <hyperlink ref="I9" r:id="rId7" display="https://kahicosmetics.co.kr/product/가히-멀티밤-리필키트-9g-x-2개/145"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1683,7 +1701,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1691,10 +1709,10 @@
         <v>10</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>